<commit_message>
Update account initialization, migrations, admin UI and database
</commit_message>
<xml_diff>
--- a/teacher-directory.xlsx
+++ b/teacher-directory.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Login@123</t>
+          <t>aPUrkycc4tuSy-gU</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">

</xml_diff>

<commit_message>
Add teacher dashboard and fix owner login
</commit_message>
<xml_diff>
--- a/teacher-directory.xlsx
+++ b/teacher-directory.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Initial Password</t>
+          <t>Initial Password (private)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -473,7 +473,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>aPUrkycc4tuSy-gU</t>
+          <t>Login@123</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">

</xml_diff>